<commit_message>
including DHF6 BAL week 21 neutrophil data typo fix
</commit_message>
<xml_diff>
--- a/input_data/ccrvb39_batch1and2_RAW_datasets.xlsx
+++ b/input_data/ccrvb39_batch1and2_RAW_datasets.xlsx
@@ -43684,31 +43684,31 @@
         <v>29.4117647058824</v>
       </c>
       <c r="O16" t="n">
-        <v>51.4705882352941</v>
+        <v>0.283673040554738</v>
       </c>
       <c r="P16" t="n">
-        <v>0.963212559661394</v>
+        <v>18.5185185185185</v>
       </c>
       <c r="Q16" t="n">
-        <v>30.453781512605</v>
+        <v>21.2962962962963</v>
       </c>
       <c r="R16" t="n">
-        <v>243.63025210084</v>
+        <v>92.5925925925926</v>
       </c>
       <c r="S16" t="n">
-        <v>126.890756302521</v>
+        <v>12.037037037037</v>
       </c>
       <c r="T16" t="n">
-        <v>167.077717407619</v>
+        <v>42.5925925925926</v>
       </c>
       <c r="U16" t="n">
-        <v>17.703085032168</v>
+        <v>12.037037037037</v>
       </c>
       <c r="V16" t="n">
-        <v>399.4167118828</v>
+        <v>82.4074074074074</v>
       </c>
       <c r="W16" t="n">
-        <v>5.8522595147663</v>
+        <v>18.5185185185185</v>
       </c>
       <c r="X16" t="n">
         <v>0.422882958604749</v>

</xml_diff>